<commit_message>
udpate - fix json and htnml files loading
</commit_message>
<xml_diff>
--- a/src/DashboardApp/pop_final.xlsx
+++ b/src/DashboardApp/pop_final.xlsx
@@ -37,151 +37,151 @@
     <t>[0, 0, 0, 0, 0]</t>
   </si>
   <si>
-    <t>[31, 28, 0, 8, 22]</t>
-  </si>
-  <si>
-    <t>[10, 12, 27, 3, 17]</t>
-  </si>
-  <si>
-    <t>[24, 16, 5, 26, 23]</t>
-  </si>
-  <si>
-    <t>[19, 27, 6, 27, 17]</t>
-  </si>
-  <si>
-    <t>[15, 15, 14, 4, 20]</t>
-  </si>
-  <si>
-    <t>[19, 23, 3, 27, 29]</t>
-  </si>
-  <si>
-    <t>[2, 7, 3, 13, 29]</t>
-  </si>
-  <si>
-    <t>[12, 4, 12, 13, 7]</t>
-  </si>
-  <si>
-    <t>[3, 23, 8, 7, 8]</t>
-  </si>
-  <si>
-    <t>[19, 17, 6, 6, 17]</t>
-  </si>
-  <si>
-    <t>[6, 20, 20, 6, 21]</t>
-  </si>
-  <si>
-    <t>[30, 6, 2, 10, 9]</t>
-  </si>
-  <si>
-    <t>[10, 0, 20, 1, 15]</t>
-  </si>
-  <si>
-    <t>[13, 10, 22, 11, 13]</t>
-  </si>
-  <si>
-    <t>[2, 1, 1, 7, 29]</t>
-  </si>
-  <si>
-    <t>[8, 29, 29, 0, 17]</t>
-  </si>
-  <si>
-    <t>[19, 23, 10, 21, 0]</t>
-  </si>
-  <si>
-    <t>[6, 23, 24, 9, 4]</t>
-  </si>
-  <si>
-    <t>[17, 12, 26, 21, 9]</t>
-  </si>
-  <si>
-    <t>[17, 25, 10, 6, 29]</t>
-  </si>
-  <si>
-    <t>[0, 13, 23, 27, 20]</t>
-  </si>
-  <si>
-    <t>[16, 12, 11, 5, 13]</t>
-  </si>
-  <si>
-    <t>[8, 8, 2, 8, 7]</t>
-  </si>
-  <si>
-    <t>[11, 14, 21, 24, 26]</t>
-  </si>
-  <si>
-    <t>[15, 28, 22, 5, 25]</t>
-  </si>
-  <si>
-    <t>[22, 8, 25, 24, 21]</t>
-  </si>
-  <si>
-    <t>[28, 30, 7, 5, 31]</t>
-  </si>
-  <si>
-    <t>[15, 12, 4, 11, 6]</t>
-  </si>
-  <si>
-    <t>[10, 31, 1, 24, 18]</t>
-  </si>
-  <si>
-    <t>[14, 31, 22, 16, 8]</t>
-  </si>
-  <si>
-    <t>[11, 14, 27, 4, 5]</t>
-  </si>
-  <si>
-    <t>[21, 27, 13, 25, 31]</t>
-  </si>
-  <si>
-    <t>[17, 30, 13, 7, 30]</t>
-  </si>
-  <si>
-    <t>[19, 10, 27, 11, 30]</t>
-  </si>
-  <si>
-    <t>[5, 29, 1, 28, 8]</t>
-  </si>
-  <si>
-    <t>[29, 15, 29, 10, 15]</t>
-  </si>
-  <si>
-    <t>[24, 14, 31, 19, 3]</t>
-  </si>
-  <si>
-    <t>[1, 30, 6, 12, 6]</t>
-  </si>
-  <si>
-    <t>[16, 18, 14, 28, 2]</t>
-  </si>
-  <si>
-    <t>[23, 20, 16, 18, 30]</t>
-  </si>
-  <si>
-    <t>[23, 9, 24, 20, 6]</t>
-  </si>
-  <si>
-    <t>[23, 18, 21, 18, 8]</t>
-  </si>
-  <si>
-    <t>[7, 27, 25, 13, 7]</t>
-  </si>
-  <si>
-    <t>[11, 22, 14, 22, 25]</t>
-  </si>
-  <si>
-    <t>[13, 29, 17, 3, 11]</t>
-  </si>
-  <si>
-    <t>[15, 19, 7, 28, 29]</t>
-  </si>
-  <si>
-    <t>[23, 4, 14, 13, 7]</t>
-  </si>
-  <si>
-    <t>[25, 16, 3, 7, 13]</t>
-  </si>
-  <si>
-    <t>[3, 28, 8, 9, 26]</t>
+    <t>[7, 26, 8, 13, 3]</t>
+  </si>
+  <si>
+    <t>[5, 0, 30, 26, 14]</t>
+  </si>
+  <si>
+    <t>[28, 5, 1, 5, 17]</t>
+  </si>
+  <si>
+    <t>[9, 30, 19, 8, 21]</t>
+  </si>
+  <si>
+    <t>[2, 4, 12, 0, 16]</t>
+  </si>
+  <si>
+    <t>[1, 2, 24, 21, 10]</t>
+  </si>
+  <si>
+    <t>[0, 5, 13, 19, 1]</t>
+  </si>
+  <si>
+    <t>[15, 6, 22, 31, 23]</t>
+  </si>
+  <si>
+    <t>[20, 7, 14, 17, 31]</t>
+  </si>
+  <si>
+    <t>[23, 21, 7, 25, 5]</t>
+  </si>
+  <si>
+    <t>[7, 3, 23, 30, 17]</t>
+  </si>
+  <si>
+    <t>[11, 31, 14, 6, 22]</t>
+  </si>
+  <si>
+    <t>[27, 7, 17, 23, 24]</t>
+  </si>
+  <si>
+    <t>[26, 4, 5, 31, 18]</t>
+  </si>
+  <si>
+    <t>[12, 12, 22, 10, 4]</t>
+  </si>
+  <si>
+    <t>[5, 26, 25, 16, 5]</t>
+  </si>
+  <si>
+    <t>[16, 25, 20, 19, 10]</t>
+  </si>
+  <si>
+    <t>[4, 6, 27, 27, 21]</t>
+  </si>
+  <si>
+    <t>[13, 7, 21, 2, 6]</t>
+  </si>
+  <si>
+    <t>[31, 10, 0, 0, 13]</t>
+  </si>
+  <si>
+    <t>[17, 19, 26, 25, 8]</t>
+  </si>
+  <si>
+    <t>[8, 24, 15, 7, 8]</t>
+  </si>
+  <si>
+    <t>[14, 19, 21, 11, 15]</t>
+  </si>
+  <si>
+    <t>[5, 18, 18, 4, 23]</t>
+  </si>
+  <si>
+    <t>[5, 31, 23, 0, 8]</t>
+  </si>
+  <si>
+    <t>[20, 26, 25, 25, 13]</t>
+  </si>
+  <si>
+    <t>[25, 18, 26, 5, 31]</t>
+  </si>
+  <si>
+    <t>[11, 22, 11, 17, 16]</t>
+  </si>
+  <si>
+    <t>[4, 16, 4, 20, 17]</t>
+  </si>
+  <si>
+    <t>[20, 25, 17, 21, 4]</t>
+  </si>
+  <si>
+    <t>[9, 26, 15, 26, 28]</t>
+  </si>
+  <si>
+    <t>[17, 10, 28, 22, 24]</t>
+  </si>
+  <si>
+    <t>[12, 7, 23, 13, 18]</t>
+  </si>
+  <si>
+    <t>[25, 23, 26, 16, 16]</t>
+  </si>
+  <si>
+    <t>[5, 0, 28, 0, 20]</t>
+  </si>
+  <si>
+    <t>[21, 11, 9, 31, 24]</t>
+  </si>
+  <si>
+    <t>[15, 29, 26, 17, 22]</t>
+  </si>
+  <si>
+    <t>[29, 31, 20, 13, 6]</t>
+  </si>
+  <si>
+    <t>[23, 13, 15, 1, 26]</t>
+  </si>
+  <si>
+    <t>[30, 9, 29, 14, 11]</t>
+  </si>
+  <si>
+    <t>[20, 19, 28, 9, 0]</t>
+  </si>
+  <si>
+    <t>[3, 18, 29, 27, 16]</t>
+  </si>
+  <si>
+    <t>[27, 9, 24, 16, 1]</t>
+  </si>
+  <si>
+    <t>[17, 18, 25, 29, 11]</t>
+  </si>
+  <si>
+    <t>[12, 23, 9, 15, 22]</t>
+  </si>
+  <si>
+    <t>[21, 23, 7, 20, 3]</t>
+  </si>
+  <si>
+    <t>[16, 24, 6, 30, 8]</t>
+  </si>
+  <si>
+    <t>[20, 27, 19, 23, 17]</t>
+  </si>
+  <si>
+    <t>[31, 13, 14, 8, 14]</t>
   </si>
   <si>
     <t>HOF</t>
@@ -602,10 +602,10 @@
         <v>7</v>
       </c>
       <c r="E3">
-        <v>2293</v>
+        <v>967</v>
       </c>
       <c r="G3">
-        <v>89</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -622,10 +622,10 @@
         <v>8</v>
       </c>
       <c r="E4">
-        <v>1271</v>
+        <v>1797</v>
       </c>
       <c r="G4">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -642,10 +642,10 @@
         <v>9</v>
       </c>
       <c r="E5">
-        <v>2062</v>
+        <v>1124</v>
       </c>
       <c r="G5">
-        <v>94</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -662,10 +662,10 @@
         <v>10</v>
       </c>
       <c r="E6">
-        <v>2144</v>
+        <v>1847</v>
       </c>
       <c r="G6">
-        <v>96</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -682,10 +682,10 @@
         <v>11</v>
       </c>
       <c r="E7">
-        <v>1062</v>
+        <v>420</v>
       </c>
       <c r="G7">
-        <v>68</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -702,10 +702,10 @@
         <v>12</v>
       </c>
       <c r="E8">
-        <v>2469</v>
+        <v>1122</v>
       </c>
       <c r="G8">
-        <v>101</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -722,10 +722,10 @@
         <v>13</v>
       </c>
       <c r="E9">
-        <v>1072</v>
+        <v>556</v>
       </c>
       <c r="G9">
-        <v>54</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -742,10 +742,10 @@
         <v>14</v>
       </c>
       <c r="E10">
-        <v>522</v>
+        <v>2235</v>
       </c>
       <c r="G10">
-        <v>48</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -762,10 +762,10 @@
         <v>15</v>
       </c>
       <c r="E11">
-        <v>715</v>
+        <v>1895</v>
       </c>
       <c r="G11">
-        <v>49</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -782,10 +782,10 @@
         <v>16</v>
       </c>
       <c r="E12">
-        <v>1011</v>
+        <v>1669</v>
       </c>
       <c r="G12">
-        <v>65</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -802,10 +802,10 @@
         <v>17</v>
       </c>
       <c r="E13">
-        <v>1313</v>
+        <v>1776</v>
       </c>
       <c r="G13">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -822,10 +822,10 @@
         <v>18</v>
       </c>
       <c r="E14">
-        <v>1121</v>
+        <v>1798</v>
       </c>
       <c r="G14">
-        <v>57</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -842,10 +842,10 @@
         <v>19</v>
       </c>
       <c r="E15">
-        <v>726</v>
+        <v>2172</v>
       </c>
       <c r="G15">
-        <v>46</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -862,10 +862,10 @@
         <v>20</v>
       </c>
       <c r="E16">
-        <v>1043</v>
+        <v>2002</v>
       </c>
       <c r="G16">
-        <v>69</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -882,10 +882,10 @@
         <v>21</v>
       </c>
       <c r="E17">
-        <v>896</v>
+        <v>888</v>
       </c>
       <c r="G17">
-        <v>40</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -902,10 +902,10 @@
         <v>22</v>
       </c>
       <c r="E18">
-        <v>2035</v>
+        <v>1607</v>
       </c>
       <c r="G18">
-        <v>83</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -922,10 +922,10 @@
         <v>23</v>
       </c>
       <c r="E19">
-        <v>1431</v>
+        <v>1742</v>
       </c>
       <c r="G19">
-        <v>73</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -942,10 +942,10 @@
         <v>24</v>
       </c>
       <c r="E20">
-        <v>1238</v>
+        <v>1951</v>
       </c>
       <c r="G20">
-        <v>66</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -962,10 +962,10 @@
         <v>25</v>
       </c>
       <c r="E21">
-        <v>1631</v>
+        <v>699</v>
       </c>
       <c r="G21">
-        <v>85</v>
+        <v>49</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -982,10 +982,10 @@
         <v>26</v>
       </c>
       <c r="E22">
-        <v>1891</v>
+        <v>1230</v>
       </c>
       <c r="G22">
-        <v>87</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1002,10 +1002,10 @@
         <v>27</v>
       </c>
       <c r="E23">
-        <v>1827</v>
+        <v>2015</v>
       </c>
       <c r="G23">
-        <v>83</v>
+        <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1022,10 +1022,10 @@
         <v>28</v>
       </c>
       <c r="E24">
-        <v>715</v>
+        <v>978</v>
       </c>
       <c r="G24">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1042,10 +1042,10 @@
         <v>29</v>
       </c>
       <c r="E25">
-        <v>245</v>
+        <v>1344</v>
       </c>
       <c r="G25">
-        <v>33</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1062,10 +1062,10 @@
         <v>30</v>
       </c>
       <c r="E26">
-        <v>2010</v>
+        <v>1218</v>
       </c>
       <c r="G26">
-        <v>96</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1082,10 +1082,10 @@
         <v>31</v>
       </c>
       <c r="E27">
-        <v>2143</v>
+        <v>1579</v>
       </c>
       <c r="G27">
-        <v>95</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1102,10 +1102,10 @@
         <v>32</v>
       </c>
       <c r="E28">
-        <v>2190</v>
+        <v>2495</v>
       </c>
       <c r="G28">
-        <v>100</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1122,10 +1122,10 @@
         <v>33</v>
       </c>
       <c r="E29">
-        <v>2719</v>
+        <v>2611</v>
       </c>
       <c r="G29">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1142,10 +1142,10 @@
         <v>34</v>
       </c>
       <c r="E30">
-        <v>542</v>
+        <v>1271</v>
       </c>
       <c r="G30">
-        <v>48</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1162,10 +1162,10 @@
         <v>35</v>
       </c>
       <c r="E31">
-        <v>1962</v>
+        <v>977</v>
       </c>
       <c r="G31">
-        <v>84</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1182,10 +1182,10 @@
         <v>36</v>
       </c>
       <c r="E32">
-        <v>1961</v>
+        <v>1771</v>
       </c>
       <c r="G32">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1202,10 +1202,10 @@
         <v>37</v>
       </c>
       <c r="E33">
-        <v>1087</v>
+        <v>2442</v>
       </c>
       <c r="G33">
-        <v>61</v>
+        <v>104</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1222,10 +1222,10 @@
         <v>38</v>
       </c>
       <c r="E34">
-        <v>2925</v>
+        <v>2233</v>
       </c>
       <c r="G34">
-        <v>117</v>
+        <v>101</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1242,10 +1242,10 @@
         <v>39</v>
       </c>
       <c r="E35">
-        <v>2307</v>
+        <v>1215</v>
       </c>
       <c r="G35">
-        <v>97</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1262,10 +1262,10 @@
         <v>40</v>
       </c>
       <c r="E36">
-        <v>2211</v>
+        <v>2342</v>
       </c>
       <c r="G36">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1282,10 +1282,10 @@
         <v>41</v>
       </c>
       <c r="E37">
-        <v>1715</v>
+        <v>1209</v>
       </c>
       <c r="G37">
-        <v>71</v>
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1302,10 +1302,10 @@
         <v>42</v>
       </c>
       <c r="E38">
-        <v>2232</v>
+        <v>2180</v>
       </c>
       <c r="G38">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1322,10 +1322,10 @@
         <v>43</v>
       </c>
       <c r="E39">
-        <v>2103</v>
+        <v>2515</v>
       </c>
       <c r="G39">
-        <v>91</v>
+        <v>109</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1342,10 +1342,10 @@
         <v>44</v>
       </c>
       <c r="E40">
-        <v>1117</v>
+        <v>2407</v>
       </c>
       <c r="G40">
-        <v>55</v>
+        <v>99</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1362,7 +1362,7 @@
         <v>45</v>
       </c>
       <c r="E41">
-        <v>1564</v>
+        <v>1600</v>
       </c>
       <c r="G41">
         <v>78</v>
@@ -1382,10 +1382,10 @@
         <v>46</v>
       </c>
       <c r="E42">
-        <v>2409</v>
+        <v>2139</v>
       </c>
       <c r="G42">
-        <v>107</v>
+        <v>93</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1402,10 +1402,10 @@
         <v>47</v>
       </c>
       <c r="E43">
-        <v>1622</v>
+        <v>1626</v>
       </c>
       <c r="G43">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1422,10 +1422,10 @@
         <v>48</v>
       </c>
       <c r="E44">
-        <v>1682</v>
+        <v>2159</v>
       </c>
       <c r="G44">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1442,10 +1442,10 @@
         <v>49</v>
       </c>
       <c r="E45">
-        <v>1621</v>
+        <v>1643</v>
       </c>
       <c r="G45">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1462,10 +1462,10 @@
         <v>50</v>
       </c>
       <c r="E46">
-        <v>1910</v>
+        <v>2200</v>
       </c>
       <c r="G46">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -1482,10 +1482,10 @@
         <v>51</v>
       </c>
       <c r="E47">
-        <v>1429</v>
+        <v>1463</v>
       </c>
       <c r="G47">
-        <v>73</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -1502,10 +1502,10 @@
         <v>52</v>
       </c>
       <c r="E48">
-        <v>2260</v>
+        <v>1428</v>
       </c>
       <c r="G48">
-        <v>98</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -1522,10 +1522,10 @@
         <v>53</v>
       </c>
       <c r="E49">
-        <v>959</v>
+        <v>1832</v>
       </c>
       <c r="G49">
-        <v>61</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -1542,10 +1542,10 @@
         <v>54</v>
       </c>
       <c r="E50">
-        <v>1108</v>
+        <v>2308</v>
       </c>
       <c r="G50">
-        <v>64</v>
+        <v>106</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -1562,10 +1562,10 @@
         <v>55</v>
       </c>
       <c r="E51">
-        <v>1614</v>
+        <v>1586</v>
       </c>
       <c r="G51">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>